<commit_message>
chore(bkm): COD raporu xlsx düzeltilmiş modelle yeniden üretildi
</commit_message>
<xml_diff>
--- a/briefings/kapida-odeme-analiz.xlsx
+++ b/briefings/kapida-odeme-analiz.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -556,12 +556,12 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>20.117</t>
+          <t>20.119</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>23.800.589 ₺</t>
+          <t>23.804.344 ₺</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -593,88 +593,95 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>• Service (kapıda ödeme) ücreti geliri: +1.707.933 ₺</t>
+          <t>• Service (kapıda ödeme) ücreti: müşteriden +1.708.103 ₺ ≈ kargo/tahsilat firmasına ödenen → NÖTR (pass-through, KÂR DEĞİL).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>• İade kargo zararı (1690 iade × 180₺ gidiş-dönüş): −304.200 ₺</t>
+          <t>• İade kargo zararı (1689 iade × 180₺ gidiş-dönüş): −304.020 ₺ (iadede tahsil de yok).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>• NET operasyonel katkı: +1.403.733 ₺</t>
+          <t>• COD NET OPERASYONEL MALİYET: −304.020 ₺ (sadece iade zararı).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr"/>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>• COD'un değeri finansal kârda değil → kartı olmayan/güvenmeyen müşteriye SATIŞ + büyük sepet (enablement). İade düştükçe maliyet düşer.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>BULGULAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>• COD iade (kapıda red) oranı %10,2 — online %0,6. COD ~17× daha riskli teslimde.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>• COD ort. sepet 1.183₺ &gt; online 970₺ → büyük sepet ama teslim riski yüksek.</t>
+          <t>• COD iade (kapıda red) oranı %10,2 — online %0,6. COD ~17× daha riskli teslimde.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>• COD ort. sepet 1.183₺ &gt; online 970₺ → büyük sepet ama teslim riski yüksek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>• Tekrar kapıda-red eden 179 müşteri (kara liste sayfası); 58'i hiç teslim almamış.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>AKSİYON</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>• Hiç teslim almayan (Teslim=0) müşterilere COD KAPAT (sadece ön ödeme).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>• ≥2 iadeli müşteriye SMS teyit zorunlu + COD limiti; 3. iadede otomatik blok.</t>
+          <t>• Hiç teslim almayan (Teslim=0) müşterilere COD KAPAT (sadece ön ödeme).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>• Misafir COD'u kısıtla (üyeye aç) — misafir takip edilemiyor.</t>
+          <t>• ≥2 iadeli müşteriye SMS teyit zorunlu + COD limiti; 3. iadede otomatik blok.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>• Misafir COD'u kısıtla (üyeye aç) — misafir takip edilemiyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>• COD iade oranını brief KPI'sına ekle (hedef &lt;%5).</t>
         </is>
@@ -748,7 +755,7 @@
         <v>14940</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>299828</v>
+        <v>299803</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>85.59999999999999</v>
@@ -761,7 +768,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>1690</v>
+        <v>1689</v>
       </c>
       <c r="C4" s="12" t="n">
         <v>1667</v>
@@ -870,16 +877,16 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>3713</v>
+        <v>3711</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>4072857</v>
+        <v>4071721</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>3172</v>
+        <v>3171</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F2" s="10" t="n">
         <v>10.9</v>
@@ -958,10 +965,10 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>1573</v>
+        <v>1577</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2093856</v>
+        <v>2098746</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>473</v>

</xml_diff>

<commit_message>
fix(bkm): COD iade zararı gerçek CARGOPRICE×2 (gidiş+geri getirme)
Flat 180 yerine veri: iade siparişlerin gerçek CARGOPRICE toplamı × 2 (götürme+
geri getirme; iadede tahsil yok, müşteri ödemez, BKM yutar). 273K (önceki tahmin 304K).
Teslim = müşteri kargo+kapıda bedeli öder → pass-through nötr.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/briefings/kapida-odeme-analiz.xlsx
+++ b/briefings/kapida-odeme-analiz.xlsx
@@ -556,12 +556,12 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>20.119</t>
+          <t>20.121</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>23.804.344 ₺</t>
+          <t>23.805.500 ₺</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -593,21 +593,21 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>• Service (kapıda ödeme) ücreti: müşteriden +1.708.103 ₺ ≈ kargo/tahsilat firmasına ödenen → NÖTR (pass-through, KÂR DEĞİL).</t>
+          <t>• Service (kapıda ödeme) ücreti: müşteriden +1.708.273 ₺ ≈ kargo/tahsilat firmasına ödenen → NÖTR (pass-through, KÂR DEĞİL).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>• İade kargo zararı (1689 iade × 180₺ gidiş-dönüş): −304.020 ₺ (iadede tahsil de yok).</t>
+          <t>• İade kargo zararı (1689 iade × gerçek kargo × 2 gidiş-dönüş = 136.501×2): −273.002 ₺ (iadede tahsil yok, müşteri ödemez).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>• COD NET OPERASYONEL MALİYET: −304.020 ₺ (sadece iade zararı).</t>
+          <t>• COD NET OPERASYONEL MALİYET: −273.002 ₺ (sadece iade zararı).</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
         <v>14940</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>299803</v>
+        <v>299795</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>85.59999999999999</v>
@@ -965,10 +965,10 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>1577</v>
+        <v>1579</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2098746</v>
+        <v>2099902</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>473</v>

</xml_diff>

<commit_message>
feat(bkm): COD raporuna İl İade + Kargo Firma (il-içi adil kıyas) sayfaları
İl bazında COD iade% (coğrafya etkisi, yüksek-risk il kırmızı + öneri) + kargo
firması genel vs İstanbul-içi iade% (coğrafyadan arındırılmış). Bulgu: iade
coğrafya kaynaklı (Doğu/GD %15-21, Batı %3-6), firma değil (İstanbul'da PTT≈HEPSIJET).
Aksiyon: firma kaydırma değil, yüksek-iade illerde COD teyit/ön-ödeme.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/briefings/kapida-odeme-analiz.xlsx
+++ b/briefings/kapida-odeme-analiz.xlsx
@@ -11,6 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teslim Performansı" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aylık Trend" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kara Liste" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="İl İade" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kargo Firma" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +69,11 @@
     <font>
       <b val="1"/>
       <color rgb="00E30622"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -113,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +139,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -561,7 +569,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>23.805.500 ₺</t>
+          <t>23.806.416 ₺</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -650,38 +658,52 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>• İade ağırlıkla COĞRAFYA kaynaklı (Doğu/GD/Karadeniz illeri %15-21, Batı %3-6) — firma DEĞİL. İstanbul-içi PTT≈HEPSIJET (Kargo Firma sayfası).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>AKSİYON</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>• Hiç teslim almayan (Teslim=0) müşterilere COD KAPAT (sadece ön ödeme).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>• ≥2 iadeli müşteriye SMS teyit zorunlu + COD limiti; 3. iadede otomatik blok.</t>
+          <t>• Yüksek-iade illerde (İl İade sayfası, %13+) COD'a ön-arama/SMS teyit veya ön-ödeme teşvik (firma kaydırma çözüm değil — HEPSIJET o illere gitmiyor).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>• Misafir COD'u kısıtla (üyeye aç) — misafir takip edilemiyor.</t>
+          <t>• Hiç teslim almayan (Teslim=0) müşterilere COD KAPAT (sadece ön ödeme).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>• ≥2 iadeli müşteriye SMS teyit zorunlu + COD limiti; 3. iadede otomatik blok.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>• Misafir COD'u kısıtla (üyeye aç) — misafir takip edilemiyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>• COD iade oranını brief KPI'sına ekle (hedef &lt;%5).</t>
         </is>
@@ -739,7 +761,7 @@
         <v>763</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>6061</v>
+        <v>6060</v>
       </c>
       <c r="D2" s="10" t="n">
         <v>4.4</v>
@@ -752,10 +774,10 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>14940</v>
+        <v>14939</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>299795</v>
+        <v>299780</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>85.59999999999999</v>
@@ -771,7 +793,7 @@
         <v>1689</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="D4" s="13" t="n">
         <v>9.699999999999999</v>
@@ -877,13 +899,13 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>3711</v>
+        <v>3710</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>4071721</v>
+        <v>4070918</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>3171</v>
+        <v>3170</v>
       </c>
       <c r="E2" s="9" t="n">
         <v>386</v>
@@ -965,10 +987,10 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2099902</v>
+        <v>2101622</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>473</v>
@@ -7320,4 +7342,1752 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>İl</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Teslim</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>İade</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>İade %</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Risk / Öneri</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Osmaniye</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="n">
+        <v>140</v>
+      </c>
+      <c r="C2" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="D2" s="17" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Trabzon</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="n">
+        <v>164</v>
+      </c>
+      <c r="C3" s="16" t="n">
+        <v>44</v>
+      </c>
+      <c r="D3" s="17" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Hakkari</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Şırnak</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>77</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Batman</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>95</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Adıyaman</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>88</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Aksaray</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>65</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Iğdır</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Ağrı</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>93</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Sakarya</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>191</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Bolu</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>51</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Erzincan</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>40</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Samsun</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>193</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Karaman</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>41</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Mardin</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>129</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>YÜKSEK — COD'a ön-arama/SMS teyit veya ön-ödeme teşvik</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Kars</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Diyarbakır</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>347</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Bingöl</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Muğla</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>230</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Çorum</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>84</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Isparta</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Tunceli</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Elazığ</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>146</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Uşak</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Kocaeli</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>298</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Karabük</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Adana</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>478</v>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Bitlis</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>64</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Şanlıurfa</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>254</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Gaziantep</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>480</v>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Ordu</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Afyonkarahisar</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>129</v>
+      </c>
+      <c r="C33" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="D33" s="10" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Kütahya</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>131</v>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>İzmir</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="n">
+        <v>824</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Tokat</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="n">
+        <v>83</v>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D36" s="10" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Erzurum</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="n">
+        <v>157</v>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="D37" s="10" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Antalya</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="n">
+        <v>582</v>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>Tekirdağ</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="n">
+        <v>224</v>
+      </c>
+      <c r="C39" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="D39" s="10" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Balıkesir</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n">
+        <v>234</v>
+      </c>
+      <c r="C40" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D40" s="10" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>Ankara</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="n">
+        <v>805</v>
+      </c>
+      <c r="C41" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="D41" s="10" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>Burdur</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D42" s="10" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>Malatya</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>154</v>
+      </c>
+      <c r="C43" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D43" s="10" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Hatay</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="n">
+        <v>475</v>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="D44" s="10" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>Kahramanmaraş</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>275</v>
+      </c>
+      <c r="C45" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="D45" s="10" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>İstanbul</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="n">
+        <v>2094</v>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>209</v>
+      </c>
+      <c r="D46" s="10" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>ORTA — izle</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>Siirt</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" s="10" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>Bursa</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="n">
+        <v>493</v>
+      </c>
+      <c r="C48" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="D48" s="10" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>Konya</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="n">
+        <v>473</v>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="D49" s="10" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>Giresun</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="n">
+        <v>104</v>
+      </c>
+      <c r="C50" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D50" s="10" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Nevşehir</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="C51" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D51" s="10" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>Zonguldak</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="n">
+        <v>105</v>
+      </c>
+      <c r="C52" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D52" s="10" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>Mersin</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="n">
+        <v>483</v>
+      </c>
+      <c r="C53" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="D53" s="10" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>Van</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="n">
+        <v>197</v>
+      </c>
+      <c r="C54" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="D54" s="10" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>Kayseri</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="n">
+        <v>202</v>
+      </c>
+      <c r="C55" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="D55" s="10" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>Aydın</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="n">
+        <v>270</v>
+      </c>
+      <c r="C56" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="D56" s="10" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>Manisa</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="n">
+        <v>308</v>
+      </c>
+      <c r="C57" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D57" s="10" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>Düzce</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="C58" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D58" s="10" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>Kilis</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="C59" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" s="10" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>Yalova</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="C60" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" s="10" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>Denizli</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="n">
+        <v>210</v>
+      </c>
+      <c r="C61" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D61" s="10" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="inlineStr">
+        <is>
+          <t>Kırıkkale</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="C62" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D62" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>Amasya</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="n">
+        <v>56</v>
+      </c>
+      <c r="C63" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D63" s="10" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>Kırşehir</t>
+        </is>
+      </c>
+      <c r="B64" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="C64" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D64" s="10" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>Yozgat</t>
+        </is>
+      </c>
+      <c r="B65" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="C65" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D65" s="10" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>Kastamonu</t>
+        </is>
+      </c>
+      <c r="B66" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="C66" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D66" s="10" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>Edirne</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="C67" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D67" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>Sivas</t>
+        </is>
+      </c>
+      <c r="B68" s="9" t="n">
+        <v>96</v>
+      </c>
+      <c r="C68" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D68" s="10" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>Kırklareli</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="n">
+        <v>97</v>
+      </c>
+      <c r="C69" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D69" s="10" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>Bilecik</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="C70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D70" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>Rize</t>
+        </is>
+      </c>
+      <c r="B71" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="C71" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D71" s="10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>Eskişehir</t>
+        </is>
+      </c>
+      <c r="B72" s="9" t="n">
+        <v>177</v>
+      </c>
+      <c r="C72" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D72" s="10" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E72" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>Çanakkale</t>
+        </is>
+      </c>
+      <c r="B73" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="C73" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D73" s="10" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
+          <t>Niğde</t>
+        </is>
+      </c>
+      <c r="B74" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="C74" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>düşük — serbest</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Kargo</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Teslim</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>İade</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Genel İade %</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>İstanbul Teslim</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>İstanbul İade</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>İstanbul İade % (adil)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>KARGOIST</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>359</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="D2" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" s="10" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>PTT KARGO</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>5298</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>677</v>
+      </c>
+      <c r="D3" s="10" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>398</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="G3" s="10" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>HEPSIJET</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>6410</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>628</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>1467</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>155</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>MNG</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>2872</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>361</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>NOT: Genel iade% yanıltıcı (PTT/MNG zor illere de gider). İstanbul-içi % adil kıyas → firma farkı küçük; iade ağırlıkla COĞRAFYA.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>